<commit_message>
Adjust ConFlux presentation label and Chinese CV publication spacing
</commit_message>
<xml_diff>
--- a/documents/papers.xlsx
+++ b/documents/papers.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R59cf61d8bf134d42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="Rcefe008db7e64a07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" r:id="Rdb60d755182248ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R9be302a8c26f448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="R258ac94c1564441a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" r:id="Re7e63552c69948b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3421,7 +3421,7 @@
         <x:v>43rd International Conference on Machine Learning (ICML 2026)</x:v>
       </x:c>
       <x:c r="K49" s="12" t="str">
-        <x:v>Oral Presentation (Top 0.7%)</x:v>
+        <x:v>Oral Presentation (0.7%)</x:v>
       </x:c>
       <x:c r="L49" s="12" t="n">
         <x:v>0</x:v>
@@ -3453,27 +3453,27 @@
         <x:v>https://icml.cc/Downloads/2026; /documents/publication/conferences/ConFlux%20-%20Multivariate%20time%20series%20in%20flux%2C%20one%20unified%20forecast%20in%20confluence.pdf</x:v>
       </x:c>
       <x:c r="AC49" s="12" t="str">
-        <x:v>Restored from repository history and the local ICML 2026 paper. Oral Presentation (Top 0.7%) retained from the original user record; not independently reverified.</x:v>
+        <x:v>Restored from repository history and the local ICML 2026 paper. Oral Presentation (0.7%) retained from the original user record; not independently reverified.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R34d13f6b28ad4981"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R6455c1a486fe4044"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R8113e1c60db44335"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="R6339fc44e0dd4ae3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="Rb45368ef03644dd5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="Re5e93fb109fb4c0a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="R9735d40a04d1483f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R6c31ddd6c84c45e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R15c4dcc9e7494136"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="Ree4f646456dc45b9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R7172534b49f24b03"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="Rc12df2a162344f8e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="Rff944a5ac23c4bab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R14495a238ec44b2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R34ce470b7cd04ecb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="R5a9af2a785fb44f3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R47b919a7d25f4052"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="Re912e7ff559d4e60"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="Re3823d0e489e42f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="Rdb7ce90e4a244602"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="R54d18a23052f437b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="Ra46012516997409a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="R750a62beb2154372"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="R0cc0d0b831dc4d61"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f7096e88e2e4c52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09d0b5921f174958"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add Shixiong Zhou and Smart Cities CAS Q2 designation
</commit_message>
<xml_diff>
--- a/documents/papers.xlsx
+++ b/documents/papers.xlsx
@@ -3021,7 +3021,9 @@
       <x:c r="L42" s="12" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M42" s="12"/>
+      <x:c r="M42" s="12">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="N42" s="12"/>
       <x:c r="O42" s="12"/>
       <x:c r="P42" s="12"/>

</xml_diff>